<commit_message>
Add links from the Chiropractors Names doc: CCSP programs, Moreau CVs, books, title rule, Zocdoc and practice pages
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/downloads/ccsp.xlsx
+++ b/downloads/ccsp.xlsx
@@ -8,7 +8,8 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Index" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Every CCSP and DACBSP, by state" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How to become a CCSP programs," sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Every CCSP and DACBSP, by state" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -35,12 +36,12 @@
       <color rgb="00FFFFFF"/>
     </font>
     <font>
+      <color rgb="001C458C"/>
+      <u val="single"/>
+    </font>
+    <font>
       <b val="1"/>
       <color rgb="001C458C"/>
-    </font>
-    <font>
-      <color rgb="001C458C"/>
-      <u val="single"/>
     </font>
   </fonts>
   <fills count="4">
@@ -77,8 +78,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -444,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -485,13 +486,28 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
+          <t>How to become a CCSP programs,</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>13</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>How to become a CCSP: programs, courses and the reading list</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
           <t>Every CCSP and DACBSP, by state</t>
         </is>
       </c>
-      <c r="B5" t="n">
+      <c r="B6" t="n">
         <v>2036</v>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>Every CCSP and DACBSP, by state (2036)</t>
         </is>
@@ -500,12 +516,369 @@
   </sheetData>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A5" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A6" r:id="rId2"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="50" customWidth="1" min="1" max="1"/>
+    <col width="48" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Offered by</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>What it is</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Every saved copy</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>American Chiropractic Board of Sports Physicians</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>CCSP and DACBSP programs</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>Wayback</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>American Chiropractic Board of Sports Physicians</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Member directory</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Wayback</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>American Chiropractic Board of Sports Physicians</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>CCSP online course, summer 2026 (PDF)</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Wayback</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>American Chiropractic Board of Sports Physicians</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>CCSP reading list (PDF)</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>Wayback</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>DC Online</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Certification programming</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>Wayback</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>DC Online</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Instructors</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>Wayback</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>National University of Health Sciences</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Online courses</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>Wayback</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>National University of Health Sciences</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>CCSP course bundle</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>Wayback</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Northeast College of Health Sciences</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>CCSP courses</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>Wayback</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Northeast College of Health Sciences</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>CCSP category</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>Wayback</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Northwestern Health Sciences University</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Chiropractic Sports Injuries, CCSP 1-9 package</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>Wayback</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Life Chiropractic College West</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Course syllabi</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>Wayback</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Palmer College of Chiropractic</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>How to become a sports chiropractor</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>Wayback</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C3" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C4" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D4" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D5" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D6" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D7" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D8" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D9" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D10" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D11" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D12" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D13" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D14" r:id="rId26"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Remove CA revenue table; label main directory table; short readable workbook tab names
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/downloads/ccsp.xlsx
+++ b/downloads/ccsp.xlsx
@@ -8,8 +8,8 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Index" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How to become a CCSP programs," sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Every CCSP and DACBSP, by state" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How to become a CCSP" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CCSP and DACBSP by state" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -486,7 +486,7 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>How to become a CCSP programs,</t>
+          <t>How to become a CCSP</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -501,7 +501,7 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Every CCSP and DACBSP, by state</t>
+          <t>CCSP and DACBSP by state</t>
         </is>
       </c>
       <c r="B6" t="n">

</xml_diff>